<commit_message>
feat: add farm offline progression and monetization bridge
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/excel/Plant.xlsx
+++ b/excel/Plant.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,11 @@
           <t>收获阅历奖励</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>基础产出</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -469,6 +474,11 @@
           <t>expReward</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>baseYield</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,6 +506,11 @@
           <t>number</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,6 +538,11 @@
           <t>client</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,6 +566,11 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>client</t>
         </is>
@@ -569,6 +594,9 @@
       <c r="E6" t="n">
         <v>10</v>
       </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -588,6 +616,9 @@
       <c r="E7" t="n">
         <v>30</v>
       </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -607,6 +638,9 @@
       <c r="E8" t="n">
         <v>80</v>
       </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -626,6 +660,9 @@
       <c r="E9" t="n">
         <v>20</v>
       </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -645,6 +682,9 @@
       <c r="E10" t="n">
         <v>50</v>
       </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -663,6 +703,9 @@
       </c>
       <c r="E11" t="n">
         <v>150</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: close farm loop with subsidies and chat broadcasts
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/excel/Plant.xlsx
+++ b/excel/Plant.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>基础产出</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>需求境界等级</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,6 +484,11 @@
           <t>baseYield</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>requireLevel</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -511,6 +521,11 @@
           <t>number</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -543,6 +558,11 @@
           <t>client</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -571,6 +591,11 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>client</t>
         </is>
@@ -597,6 +622,9 @@
       <c r="F6" t="n">
         <v>1</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -619,6 +647,9 @@
       <c r="F7" t="n">
         <v>1</v>
       </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -641,6 +672,9 @@
       <c r="F8" t="n">
         <v>1</v>
       </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -663,6 +697,9 @@
       <c r="F9" t="n">
         <v>1</v>
       </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -685,6 +722,9 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -706,6 +746,9 @@
       </c>
       <c r="F11" t="n">
         <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>